<commit_message>
cleaning up visuals and repo
</commit_message>
<xml_diff>
--- a/Chanthadara_territory_chart.xlsx
+++ b/Chanthadara_territory_chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chimm\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEDA2E0A-1B2D-4AEC-A129-44F09A8AC823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{16DC384D-B764-4646-A005-A43770CCC189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4F9622DB-3F0B-4399-96EC-3CBDB6BB25F8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{4F9622DB-3F0B-4399-96EC-3CBDB6BB25F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Findings" sheetId="7" r:id="rId1"/>

</xml_diff>